<commit_message>
chore: Addresabble 전 데이터 테이블 수정
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/InteractableContainer.xlsx
+++ b/JsonConverter/ExcelFiles/InteractableContainer.xlsx
@@ -198,13 +198,13 @@
     <t>0,10,50,40</t>
   </si>
   <si>
+    <t>망가진 금고</t>
+  </si>
+  <si>
+    <t>0,40,50,10</t>
+  </si>
+  <si>
     <t>Mesh_BrokenIronBox_Prefab</t>
-  </si>
-  <si>
-    <t>망가진 금고</t>
-  </si>
-  <si>
-    <t>0,40,50,10</t>
   </si>
   <si>
     <t>Object_06</t>
@@ -987,7 +987,7 @@
         <v>5.0</v>
       </c>
       <c r="M7" s="20" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -995,7 +995,7 @@
         <v>55</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>37</v>
@@ -1018,13 +1018,13 @@
         <v>39</v>
       </c>
       <c r="K8" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L8" s="20">
         <v>1.0</v>
       </c>
       <c r="M8" s="20" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
fix: Enemy가 문에 부딪히는 경우에서 시간과 거리 조금 더 줄이고, InteractableContainer와 PreLoadAsset 최신화 (기준: 06/29 21:17)
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/InteractableContainer.xlsx
+++ b/JsonConverter/ExcelFiles/InteractableContainer.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="68">
   <si>
     <t>데이터 Id</t>
   </si>
@@ -198,13 +198,13 @@
     <t>0,10,50,40</t>
   </si>
   <si>
+    <t>망가진 금고</t>
+  </si>
+  <si>
+    <t>0,40,50,10</t>
+  </si>
+  <si>
     <t>Mesh_BrokenIronBox_Prefab</t>
-  </si>
-  <si>
-    <t>망가진 금고</t>
-  </si>
-  <si>
-    <t>0,40,50,10</t>
   </si>
   <si>
     <t>Object_06</t>
@@ -246,7 +246,7 @@
       <name val="&quot;\0022맑은 고딕\0022&quot;"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -259,6 +259,12 @@
         <bgColor theme="0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="16">
     <border/>
@@ -419,7 +425,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -488,6 +494,21 @@
     </xf>
     <xf borderId="7" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="15" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="15" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="7" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="7" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -987,7 +1008,7 @@
         <v>5.0</v>
       </c>
       <c r="M7" s="20" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -995,7 +1016,7 @@
         <v>55</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>37</v>
@@ -1018,49 +1039,49 @@
         <v>39</v>
       </c>
       <c r="K8" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L8" s="20">
         <v>1.0</v>
       </c>
       <c r="M8" s="20" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="23" t="s">
         <v>65</v>
       </c>
       <c r="E9" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="J9" s="20" t="s">
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="24">
+        <v>0.0</v>
+      </c>
+      <c r="J9" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="K9" s="20" t="s">
+      <c r="K9" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="20">
+      <c r="L9" s="27">
         <v>1.0</v>
       </c>
-      <c r="M9" s="20" t="s">
+      <c r="M9" s="26" t="s">
         <v>67</v>
       </c>
     </row>

</xml_diff>